<commit_message>
Fixing percentage values by removing the *100 part as it distorts the spreadsheet number formatting.
</commit_message>
<xml_diff>
--- a/PythonScripts/Grand_Tokaj_Zártkörűen_Működő_Részvénytársaság_Beszamolo_Elemzes.xlsx
+++ b/PythonScripts/Grand_Tokaj_Zártkörűen_Működő_Részvénytársaság_Beszamolo_Elemzes.xlsx
@@ -7306,31 +7306,31 @@
       </c>
       <c r="B187" t="inlineStr"/>
       <c r="C187" t="n">
-        <v>0.5689867058939813</v>
+        <v>0.005689867058939813</v>
       </c>
       <c r="D187" t="n">
-        <v>9.229044507623696</v>
+        <v>0.09229044507623696</v>
       </c>
       <c r="E187" t="n">
-        <v>-8.123039607107829</v>
+        <v>-0.08123039607107829</v>
       </c>
       <c r="F187" t="n">
-        <v>-4.855709974759925</v>
+        <v>-0.04855709974759925</v>
       </c>
       <c r="G187" t="n">
-        <v>-3.622717602493175</v>
+        <v>-0.03622717602493175</v>
       </c>
       <c r="H187" t="n">
-        <v>-1.154808440595878</v>
+        <v>-0.01154808440595878</v>
       </c>
       <c r="I187" t="n">
-        <v>-4.668003384132358</v>
+        <v>-0.04668003384132358</v>
       </c>
       <c r="J187" t="n">
-        <v>-1.876415179094182</v>
+        <v>-0.01876415179094182</v>
       </c>
       <c r="K187" t="n">
-        <v>-4.020074375666005</v>
+        <v>-0.04020074375666005</v>
       </c>
     </row>
     <row r="188">
@@ -7343,31 +7343,31 @@
         <v>0</v>
       </c>
       <c r="C188" t="n">
-        <v>0.5689867058939813</v>
+        <v>0.005689867058939813</v>
       </c>
       <c r="D188" t="n">
-        <v>4.809609888524569</v>
+        <v>0.04809609888524569</v>
       </c>
       <c r="E188" t="n">
-        <v>0.3081627527095732</v>
+        <v>0.003081627527095732</v>
       </c>
       <c r="F188" t="n">
-        <v>-1.008503579865427</v>
+        <v>-0.01008503579865427</v>
       </c>
       <c r="G188" t="n">
-        <v>-1.536958539094435</v>
+        <v>-0.01536958539094435</v>
       </c>
       <c r="H188" t="n">
-        <v>-1.473369611198139</v>
+        <v>-0.01473369611198139</v>
       </c>
       <c r="I188" t="n">
-        <v>-1.936217998462419</v>
+        <v>-0.01936217998462419</v>
       </c>
       <c r="J188" t="n">
-        <v>-1.928744639729696</v>
+        <v>-0.01928744639729696</v>
       </c>
       <c r="K188" t="n">
-        <v>-2.163346952042178</v>
+        <v>-0.02163346952042178</v>
       </c>
     </row>
     <row r="189">
@@ -7377,34 +7377,34 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>39.67460916372919</v>
+        <v>0.3967460916372919</v>
       </c>
       <c r="C189" t="n">
-        <v>48.0559631573108</v>
+        <v>0.480559631573108</v>
       </c>
       <c r="D189" t="n">
-        <v>49.42677125986611</v>
+        <v>0.4942677125986611</v>
       </c>
       <c r="E189" t="n">
-        <v>97.17870388325558</v>
+        <v>0.9717870388325558</v>
       </c>
       <c r="F189" t="n">
-        <v>96.38866593637221</v>
+        <v>0.9638866593637221</v>
       </c>
       <c r="G189" t="n">
-        <v>94.25982906878335</v>
+        <v>0.9425982906878335</v>
       </c>
       <c r="H189" t="n">
-        <v>91.68978912082477</v>
+        <v>0.9168978912082477</v>
       </c>
       <c r="I189" t="n">
-        <v>91.45710165941881</v>
+        <v>0.914571016594188</v>
       </c>
       <c r="J189" t="n">
-        <v>91.13472507337876</v>
+        <v>0.9113472507337876</v>
       </c>
       <c r="K189" t="n">
-        <v>92.13454863499433</v>
+        <v>0.9213454863499433</v>
       </c>
     </row>
     <row r="190">
@@ -7414,34 +7414,34 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>52.48114187675067</v>
+        <v>0.5248114187675067</v>
       </c>
       <c r="C190" t="n">
-        <v>44.14416809939558</v>
+        <v>0.4414416809939558</v>
       </c>
       <c r="D190" t="n">
-        <v>50.49335738845949</v>
+        <v>0.5049335738845949</v>
       </c>
       <c r="E190" t="n">
-        <v>2.82129611674442</v>
+        <v>0.0282129611674442</v>
       </c>
       <c r="F190" t="n">
-        <v>3.611334063627794</v>
+        <v>0.03611334063627794</v>
       </c>
       <c r="G190" t="n">
-        <v>5.740170931216648</v>
+        <v>0.05740170931216648</v>
       </c>
       <c r="H190" t="n">
-        <v>8.310210879175226</v>
+        <v>0.08310210879175227</v>
       </c>
       <c r="I190" t="n">
-        <v>8.542898340581189</v>
+        <v>0.0854289834058119</v>
       </c>
       <c r="J190" t="n">
-        <v>8.865274926621236</v>
+        <v>0.08865274926621236</v>
       </c>
       <c r="K190" t="n">
-        <v>7.865451365005676</v>
+        <v>0.07865451365005675</v>
       </c>
     </row>
     <row r="191">
@@ -7451,34 +7451,34 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>92.15575104047986</v>
+        <v>0.9215575104047986</v>
       </c>
       <c r="C191" t="n">
-        <v>92.20013125670638</v>
+        <v>0.9220013125670639</v>
       </c>
       <c r="D191" t="n">
-        <v>99.9201286483256</v>
+        <v>0.999201286483256</v>
       </c>
       <c r="E191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="H191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="J191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="K191" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -7488,34 +7488,34 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>132.2789133477572</v>
+        <v>1.322789133477572</v>
       </c>
       <c r="C192" t="n">
-        <v>91.85991747765</v>
+        <v>0.9185991747765</v>
       </c>
       <c r="D192" t="n">
-        <v>102.1579117984173</v>
+        <v>1.021579117984173</v>
       </c>
       <c r="E192" t="n">
-        <v>2.903204101316014</v>
+        <v>0.02903204101316014</v>
       </c>
       <c r="F192" t="n">
-        <v>3.746637665897043</v>
+        <v>0.03746637665897043</v>
       </c>
       <c r="G192" t="n">
-        <v>6.089731954667482</v>
+        <v>0.06089731954667482</v>
       </c>
       <c r="H192" t="n">
-        <v>9.063398398947561</v>
+        <v>0.0906339839894756</v>
       </c>
       <c r="I192" t="n">
-        <v>9.340880243936082</v>
+        <v>0.09340880243936082</v>
       </c>
       <c r="J192" t="n">
-        <v>9.727658605962986</v>
+        <v>0.09727658605962985</v>
       </c>
       <c r="K192" t="n">
-        <v>8.536918540911199</v>
+        <v>0.08536918540911198</v>
       </c>
     </row>
     <row r="193">
@@ -7525,34 +7525,34 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>133.9873195437993</v>
+        <v>1.339873195437993</v>
       </c>
       <c r="C193" t="n">
-        <v>156.9972288051858</v>
+        <v>1.569972288051858</v>
       </c>
       <c r="D193" t="n">
-        <v>174.1658765870567</v>
+        <v>1.741658765870567</v>
       </c>
       <c r="E193" t="n">
-        <v>313.0440186276809</v>
+        <v>3.13044018627681</v>
       </c>
       <c r="F193" t="n">
-        <v>295.422117625919</v>
+        <v>2.95422117625919</v>
       </c>
       <c r="G193" t="n">
-        <v>278.4314963538261</v>
+        <v>2.784314963538261</v>
       </c>
       <c r="H193" t="n">
-        <v>267.7122442562155</v>
+        <v>2.677122442562155</v>
       </c>
       <c r="I193" t="n">
-        <v>254.5677499538301</v>
+        <v>2.545677499538301</v>
       </c>
       <c r="J193" t="n">
-        <v>248.9105152560308</v>
+        <v>2.489105152560308</v>
       </c>
       <c r="K193" t="n">
-        <v>241.525103944656</v>
+        <v>2.41525103944656</v>
       </c>
     </row>
     <row r="194">
@@ -7563,31 +7563,31 @@
       </c>
       <c r="B194" t="inlineStr"/>
       <c r="C194" t="n">
-        <v>23.00990926138644</v>
+        <v>0.2300990926138644</v>
       </c>
       <c r="D194" t="n">
-        <v>17.16864778187099</v>
+        <v>0.1716864778187097</v>
       </c>
       <c r="E194" t="n">
-        <v>138.8781420406242</v>
+        <v>1.388781420406242</v>
       </c>
       <c r="F194" t="n">
-        <v>-17.6219010017619</v>
+        <v>-0.1762190100176193</v>
       </c>
       <c r="G194" t="n">
-        <v>-16.99062127209294</v>
+        <v>-0.1699062127209294</v>
       </c>
       <c r="H194" t="n">
-        <v>-10.71925209761065</v>
+        <v>-0.1071925209761062</v>
       </c>
       <c r="I194" t="n">
-        <v>-13.14449430238537</v>
+        <v>-0.1314449430238538</v>
       </c>
       <c r="J194" t="n">
-        <v>-5.657234697799311</v>
+        <v>-0.05657234697799307</v>
       </c>
       <c r="K194" t="n">
-        <v>-7.385411311374753</v>
+        <v>-0.07385411311374757</v>
       </c>
     </row>
     <row r="195">
@@ -7597,34 +7597,34 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>67.77282905813377</v>
+        <v>0.6777282905813377</v>
       </c>
       <c r="C195" t="n">
-        <v>85.45617766628563</v>
+        <v>0.8545617766628563</v>
       </c>
       <c r="D195" t="n">
-        <v>100.1479455713752</v>
+        <v>1.001479455713752</v>
       </c>
       <c r="E195" t="n">
-        <v>174.4103502546392</v>
+        <v>1.744103502546392</v>
       </c>
       <c r="F195" t="n">
-        <v>172.8951683682732</v>
+        <v>1.728951683682732</v>
       </c>
       <c r="G195" t="n">
-        <v>164.3857251807618</v>
+        <v>1.643857251807618</v>
       </c>
       <c r="H195" t="n">
-        <v>161.7608033490167</v>
+        <v>1.617608033490167</v>
       </c>
       <c r="I195" t="n">
-        <v>158.1964441855495</v>
+        <v>1.581964441855495</v>
       </c>
       <c r="J195" t="n">
-        <v>160.1761799141536</v>
+        <v>1.601761799141536</v>
       </c>
       <c r="K195" t="n">
-        <v>158.6712023003454</v>
+        <v>1.586712023003454</v>
       </c>
     </row>
     <row r="196">
@@ -7634,34 +7634,34 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>133.3885639830715</v>
+        <v>1.333885639830715</v>
       </c>
       <c r="C196" t="n">
-        <v>156.1803346866136</v>
+        <v>1.561803346866136</v>
       </c>
       <c r="D196" t="n">
-        <v>100.1479455713752</v>
+        <v>1.001479455713752</v>
       </c>
       <c r="E196" t="n">
-        <v>174.4103502546392</v>
+        <v>1.744103502546392</v>
       </c>
       <c r="F196" t="n">
-        <v>172.8951683682732</v>
+        <v>1.728951683682732</v>
       </c>
       <c r="G196" t="n">
-        <v>164.3857251807618</v>
+        <v>1.643857251807618</v>
       </c>
       <c r="H196" t="n">
-        <v>161.9021150613012</v>
+        <v>1.619021150613012</v>
       </c>
       <c r="I196" t="n">
-        <v>158.1964441855495</v>
+        <v>1.581964441855495</v>
       </c>
       <c r="J196" t="n">
-        <v>160.1761799141536</v>
+        <v>1.601761799141536</v>
       </c>
       <c r="K196" t="n">
-        <v>158.6712023003454</v>
+        <v>1.586712023003454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Started work on a batch corporate financial record processor.
</commit_message>
<xml_diff>
--- a/PythonScripts/Grand_Tokaj_Zártkörűen_Működő_Részvénytársaság_Beszamolo_Elemzes.xlsx
+++ b/PythonScripts/Grand_Tokaj_Zártkörűen_Működő_Részvénytársaság_Beszamolo_Elemzes.xlsx
@@ -7306,31 +7306,31 @@
       </c>
       <c r="B187" t="inlineStr"/>
       <c r="C187" t="n">
-        <v>0.005689867058939813</v>
+        <v>0.5689867058939813</v>
       </c>
       <c r="D187" t="n">
-        <v>0.09229044507623696</v>
+        <v>9.229044507623696</v>
       </c>
       <c r="E187" t="n">
-        <v>-0.08123039607107829</v>
+        <v>-8.123039607107829</v>
       </c>
       <c r="F187" t="n">
-        <v>-0.04855709974759925</v>
+        <v>-4.855709974759925</v>
       </c>
       <c r="G187" t="n">
-        <v>-0.03622717602493175</v>
+        <v>-3.622717602493175</v>
       </c>
       <c r="H187" t="n">
-        <v>-0.01154808440595878</v>
+        <v>-1.154808440595878</v>
       </c>
       <c r="I187" t="n">
-        <v>-0.04668003384132358</v>
+        <v>-4.668003384132358</v>
       </c>
       <c r="J187" t="n">
-        <v>-0.01876415179094182</v>
+        <v>-1.876415179094182</v>
       </c>
       <c r="K187" t="n">
-        <v>-0.04020074375666005</v>
+        <v>-4.020074375666005</v>
       </c>
     </row>
     <row r="188">
@@ -7343,31 +7343,31 @@
         <v>0</v>
       </c>
       <c r="C188" t="n">
-        <v>0.005689867058939813</v>
+        <v>0.5689867058939813</v>
       </c>
       <c r="D188" t="n">
-        <v>0.04809609888524569</v>
+        <v>4.809609888524569</v>
       </c>
       <c r="E188" t="n">
-        <v>0.003081627527095732</v>
+        <v>0.3081627527095732</v>
       </c>
       <c r="F188" t="n">
-        <v>-0.01008503579865427</v>
+        <v>-1.008503579865427</v>
       </c>
       <c r="G188" t="n">
-        <v>-0.01536958539094435</v>
+        <v>-1.536958539094435</v>
       </c>
       <c r="H188" t="n">
-        <v>-0.01473369611198139</v>
+        <v>-1.473369611198139</v>
       </c>
       <c r="I188" t="n">
-        <v>-0.01936217998462419</v>
+        <v>-1.936217998462419</v>
       </c>
       <c r="J188" t="n">
-        <v>-0.01928744639729696</v>
+        <v>-1.928744639729696</v>
       </c>
       <c r="K188" t="n">
-        <v>-0.02163346952042178</v>
+        <v>-2.163346952042178</v>
       </c>
     </row>
     <row r="189">
@@ -7377,34 +7377,34 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0.3967460916372919</v>
+        <v>39.67460916372919</v>
       </c>
       <c r="C189" t="n">
-        <v>0.480559631573108</v>
+        <v>48.0559631573108</v>
       </c>
       <c r="D189" t="n">
-        <v>0.4942677125986611</v>
+        <v>49.42677125986611</v>
       </c>
       <c r="E189" t="n">
-        <v>0.9717870388325558</v>
+        <v>97.17870388325558</v>
       </c>
       <c r="F189" t="n">
-        <v>0.9638866593637221</v>
+        <v>96.38866593637221</v>
       </c>
       <c r="G189" t="n">
-        <v>0.9425982906878335</v>
+        <v>94.25982906878335</v>
       </c>
       <c r="H189" t="n">
-        <v>0.9168978912082477</v>
+        <v>91.68978912082477</v>
       </c>
       <c r="I189" t="n">
-        <v>0.914571016594188</v>
+        <v>91.45710165941881</v>
       </c>
       <c r="J189" t="n">
-        <v>0.9113472507337876</v>
+        <v>91.13472507337876</v>
       </c>
       <c r="K189" t="n">
-        <v>0.9213454863499433</v>
+        <v>92.13454863499433</v>
       </c>
     </row>
     <row r="190">
@@ -7414,34 +7414,34 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>0.5248114187675067</v>
+        <v>52.48114187675067</v>
       </c>
       <c r="C190" t="n">
-        <v>0.4414416809939558</v>
+        <v>44.14416809939558</v>
       </c>
       <c r="D190" t="n">
-        <v>0.5049335738845949</v>
+        <v>50.49335738845949</v>
       </c>
       <c r="E190" t="n">
-        <v>0.0282129611674442</v>
+        <v>2.82129611674442</v>
       </c>
       <c r="F190" t="n">
-        <v>0.03611334063627794</v>
+        <v>3.611334063627794</v>
       </c>
       <c r="G190" t="n">
-        <v>0.05740170931216648</v>
+        <v>5.740170931216648</v>
       </c>
       <c r="H190" t="n">
-        <v>0.08310210879175227</v>
+        <v>8.310210879175226</v>
       </c>
       <c r="I190" t="n">
-        <v>0.0854289834058119</v>
+        <v>8.542898340581189</v>
       </c>
       <c r="J190" t="n">
-        <v>0.08865274926621236</v>
+        <v>8.865274926621236</v>
       </c>
       <c r="K190" t="n">
-        <v>0.07865451365005675</v>
+        <v>7.865451365005676</v>
       </c>
     </row>
     <row r="191">
@@ -7451,34 +7451,34 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>0.9215575104047986</v>
+        <v>92.15575104047986</v>
       </c>
       <c r="C191" t="n">
-        <v>0.9220013125670639</v>
+        <v>92.20013125670638</v>
       </c>
       <c r="D191" t="n">
-        <v>0.999201286483256</v>
+        <v>99.9201286483256</v>
       </c>
       <c r="E191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="H191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="J191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="K191" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="192">
@@ -7488,34 +7488,34 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>1.322789133477572</v>
+        <v>132.2789133477572</v>
       </c>
       <c r="C192" t="n">
-        <v>0.9185991747765</v>
+        <v>91.85991747765</v>
       </c>
       <c r="D192" t="n">
-        <v>1.021579117984173</v>
+        <v>102.1579117984173</v>
       </c>
       <c r="E192" t="n">
-        <v>0.02903204101316014</v>
+        <v>2.903204101316014</v>
       </c>
       <c r="F192" t="n">
-        <v>0.03746637665897043</v>
+        <v>3.746637665897043</v>
       </c>
       <c r="G192" t="n">
-        <v>0.06089731954667482</v>
+        <v>6.089731954667482</v>
       </c>
       <c r="H192" t="n">
-        <v>0.0906339839894756</v>
+        <v>9.063398398947561</v>
       </c>
       <c r="I192" t="n">
-        <v>0.09340880243936082</v>
+        <v>9.340880243936082</v>
       </c>
       <c r="J192" t="n">
-        <v>0.09727658605962985</v>
+        <v>9.727658605962986</v>
       </c>
       <c r="K192" t="n">
-        <v>0.08536918540911198</v>
+        <v>8.536918540911199</v>
       </c>
     </row>
     <row r="193">
@@ -7525,34 +7525,34 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>1.339873195437993</v>
+        <v>133.9873195437993</v>
       </c>
       <c r="C193" t="n">
-        <v>1.569972288051858</v>
+        <v>156.9972288051858</v>
       </c>
       <c r="D193" t="n">
-        <v>1.741658765870567</v>
+        <v>174.1658765870567</v>
       </c>
       <c r="E193" t="n">
-        <v>3.13044018627681</v>
+        <v>313.0440186276809</v>
       </c>
       <c r="F193" t="n">
-        <v>2.95422117625919</v>
+        <v>295.422117625919</v>
       </c>
       <c r="G193" t="n">
-        <v>2.784314963538261</v>
+        <v>278.4314963538261</v>
       </c>
       <c r="H193" t="n">
-        <v>2.677122442562155</v>
+        <v>267.7122442562155</v>
       </c>
       <c r="I193" t="n">
-        <v>2.545677499538301</v>
+        <v>254.5677499538301</v>
       </c>
       <c r="J193" t="n">
-        <v>2.489105152560308</v>
+        <v>248.9105152560308</v>
       </c>
       <c r="K193" t="n">
-        <v>2.41525103944656</v>
+        <v>241.525103944656</v>
       </c>
     </row>
     <row r="194">
@@ -7563,31 +7563,31 @@
       </c>
       <c r="B194" t="inlineStr"/>
       <c r="C194" t="n">
-        <v>0.2300990926138644</v>
+        <v>23.00990926138644</v>
       </c>
       <c r="D194" t="n">
-        <v>0.1716864778187097</v>
+        <v>17.16864778187099</v>
       </c>
       <c r="E194" t="n">
-        <v>1.388781420406242</v>
+        <v>138.8781420406242</v>
       </c>
       <c r="F194" t="n">
-        <v>-0.1762190100176193</v>
+        <v>-17.6219010017619</v>
       </c>
       <c r="G194" t="n">
-        <v>-0.1699062127209294</v>
+        <v>-16.99062127209294</v>
       </c>
       <c r="H194" t="n">
-        <v>-0.1071925209761062</v>
+        <v>-10.71925209761065</v>
       </c>
       <c r="I194" t="n">
-        <v>-0.1314449430238538</v>
+        <v>-13.14449430238537</v>
       </c>
       <c r="J194" t="n">
-        <v>-0.05657234697799307</v>
+        <v>-5.657234697799311</v>
       </c>
       <c r="K194" t="n">
-        <v>-0.07385411311374757</v>
+        <v>-7.385411311374753</v>
       </c>
     </row>
     <row r="195">
@@ -7597,34 +7597,34 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>0.6777282905813377</v>
+        <v>67.77282905813377</v>
       </c>
       <c r="C195" t="n">
-        <v>0.8545617766628563</v>
+        <v>85.45617766628563</v>
       </c>
       <c r="D195" t="n">
-        <v>1.001479455713752</v>
+        <v>100.1479455713752</v>
       </c>
       <c r="E195" t="n">
-        <v>1.744103502546392</v>
+        <v>174.4103502546392</v>
       </c>
       <c r="F195" t="n">
-        <v>1.728951683682732</v>
+        <v>172.8951683682732</v>
       </c>
       <c r="G195" t="n">
-        <v>1.643857251807618</v>
+        <v>164.3857251807618</v>
       </c>
       <c r="H195" t="n">
-        <v>1.617608033490167</v>
+        <v>161.7608033490167</v>
       </c>
       <c r="I195" t="n">
-        <v>1.581964441855495</v>
+        <v>158.1964441855495</v>
       </c>
       <c r="J195" t="n">
-        <v>1.601761799141536</v>
+        <v>160.1761799141536</v>
       </c>
       <c r="K195" t="n">
-        <v>1.586712023003454</v>
+        <v>158.6712023003454</v>
       </c>
     </row>
     <row r="196">
@@ -7634,34 +7634,34 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>1.333885639830715</v>
+        <v>133.3885639830715</v>
       </c>
       <c r="C196" t="n">
-        <v>1.561803346866136</v>
+        <v>156.1803346866136</v>
       </c>
       <c r="D196" t="n">
-        <v>1.001479455713752</v>
+        <v>100.1479455713752</v>
       </c>
       <c r="E196" t="n">
-        <v>1.744103502546392</v>
+        <v>174.4103502546392</v>
       </c>
       <c r="F196" t="n">
-        <v>1.728951683682732</v>
+        <v>172.8951683682732</v>
       </c>
       <c r="G196" t="n">
-        <v>1.643857251807618</v>
+        <v>164.3857251807618</v>
       </c>
       <c r="H196" t="n">
-        <v>1.619021150613012</v>
+        <v>161.9021150613012</v>
       </c>
       <c r="I196" t="n">
-        <v>1.581964441855495</v>
+        <v>158.1964441855495</v>
       </c>
       <c r="J196" t="n">
-        <v>1.601761799141536</v>
+        <v>160.1761799141536</v>
       </c>
       <c r="K196" t="n">
-        <v>1.586712023003454</v>
+        <v>158.6712023003454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>